<commit_message>
Correccion de días en la gantt
</commit_message>
<xml_diff>
--- a/Schedule/Carta Gantt.xlsx
+++ b/Schedule/Carta Gantt.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Descargas\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ignac\Desktop\Bidirectional-Buck-DC-DC-converter\Schedule\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{920A9483-5C17-452B-85CD-77C0ED25E3BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8FA59880-1427-4C54-8444-BF6AED2976EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="360" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja 1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="239" uniqueCount="87">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="239" uniqueCount="88">
   <si>
     <t>Taller de sistemas electrónicos</t>
   </si>
@@ -300,6 +300,9 @@
     <t>Integrantes: Agustín Torres Bobadilla
                       Gian Lucas Barbagelata 
                        Ignacio Cerda Torres</t>
+  </si>
+  <si>
+    <t>Agustín Torres e Ignacio Cerda</t>
   </si>
 </sst>
 </file>
@@ -905,19 +908,6 @@
     </xf>
     <xf numFmtId="0" fontId="14" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="164" fontId="14" fillId="10" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="14" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="16" fillId="22" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="22" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="18" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -968,6 +958,19 @@
     <xf numFmtId="0" fontId="4" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="14" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1221,63 +1224,63 @@
       <c r="E3" s="3"/>
       <c r="F3" s="4"/>
       <c r="G3" s="4"/>
-      <c r="H3" s="81"/>
-      <c r="I3" s="82"/>
-      <c r="J3" s="82"/>
-      <c r="K3" s="81"/>
-      <c r="L3" s="82"/>
-      <c r="M3" s="82"/>
-      <c r="N3" s="81"/>
-      <c r="O3" s="82"/>
-      <c r="P3" s="82"/>
-      <c r="Q3" s="81"/>
-      <c r="R3" s="82"/>
-      <c r="S3" s="82"/>
-      <c r="T3" s="81"/>
-      <c r="U3" s="82"/>
-      <c r="V3" s="82"/>
-      <c r="W3" s="81"/>
-      <c r="X3" s="82"/>
-      <c r="Y3" s="82"/>
-      <c r="Z3" s="81"/>
-      <c r="AA3" s="82"/>
-      <c r="AB3" s="82"/>
-      <c r="AC3" s="81"/>
-      <c r="AD3" s="82"/>
-      <c r="AE3" s="82"/>
-      <c r="AF3" s="81"/>
-      <c r="AG3" s="82"/>
-      <c r="AH3" s="82"/>
-      <c r="AI3" s="81"/>
-      <c r="AJ3" s="82"/>
-      <c r="AK3" s="82"/>
-      <c r="AL3" s="81"/>
-      <c r="AM3" s="82"/>
-      <c r="AN3" s="82"/>
-      <c r="AO3" s="81"/>
-      <c r="AP3" s="82"/>
-      <c r="AQ3" s="82"/>
-      <c r="AR3" s="81"/>
-      <c r="AS3" s="82"/>
-      <c r="AT3" s="82"/>
-      <c r="AU3" s="81"/>
-      <c r="AV3" s="82"/>
-      <c r="AW3" s="82"/>
-      <c r="AX3" s="81"/>
-      <c r="AY3" s="82"/>
-      <c r="AZ3" s="82"/>
-      <c r="BA3" s="81"/>
-      <c r="BB3" s="82"/>
-      <c r="BC3" s="82"/>
-      <c r="BD3" s="81"/>
-      <c r="BE3" s="82"/>
-      <c r="BF3" s="82"/>
-      <c r="BG3" s="81"/>
-      <c r="BH3" s="82"/>
-      <c r="BI3" s="82"/>
-      <c r="BJ3" s="81"/>
-      <c r="BK3" s="82"/>
-      <c r="BL3" s="82"/>
+      <c r="H3" s="101"/>
+      <c r="I3" s="102"/>
+      <c r="J3" s="102"/>
+      <c r="K3" s="101"/>
+      <c r="L3" s="102"/>
+      <c r="M3" s="102"/>
+      <c r="N3" s="101"/>
+      <c r="O3" s="102"/>
+      <c r="P3" s="102"/>
+      <c r="Q3" s="101"/>
+      <c r="R3" s="102"/>
+      <c r="S3" s="102"/>
+      <c r="T3" s="101"/>
+      <c r="U3" s="102"/>
+      <c r="V3" s="102"/>
+      <c r="W3" s="101"/>
+      <c r="X3" s="102"/>
+      <c r="Y3" s="102"/>
+      <c r="Z3" s="101"/>
+      <c r="AA3" s="102"/>
+      <c r="AB3" s="102"/>
+      <c r="AC3" s="101"/>
+      <c r="AD3" s="102"/>
+      <c r="AE3" s="102"/>
+      <c r="AF3" s="101"/>
+      <c r="AG3" s="102"/>
+      <c r="AH3" s="102"/>
+      <c r="AI3" s="101"/>
+      <c r="AJ3" s="102"/>
+      <c r="AK3" s="102"/>
+      <c r="AL3" s="101"/>
+      <c r="AM3" s="102"/>
+      <c r="AN3" s="102"/>
+      <c r="AO3" s="101"/>
+      <c r="AP3" s="102"/>
+      <c r="AQ3" s="102"/>
+      <c r="AR3" s="101"/>
+      <c r="AS3" s="102"/>
+      <c r="AT3" s="102"/>
+      <c r="AU3" s="101"/>
+      <c r="AV3" s="102"/>
+      <c r="AW3" s="102"/>
+      <c r="AX3" s="101"/>
+      <c r="AY3" s="102"/>
+      <c r="AZ3" s="102"/>
+      <c r="BA3" s="101"/>
+      <c r="BB3" s="102"/>
+      <c r="BC3" s="102"/>
+      <c r="BD3" s="101"/>
+      <c r="BE3" s="102"/>
+      <c r="BF3" s="102"/>
+      <c r="BG3" s="101"/>
+      <c r="BH3" s="102"/>
+      <c r="BI3" s="102"/>
+      <c r="BJ3" s="101"/>
+      <c r="BK3" s="102"/>
+      <c r="BL3" s="102"/>
       <c r="BM3" s="5"/>
       <c r="BN3" s="5"/>
       <c r="BO3" s="5"/>
@@ -1342,63 +1345,63 @@
       <c r="E4" s="5"/>
       <c r="F4" s="7"/>
       <c r="G4" s="5"/>
-      <c r="H4" s="81"/>
-      <c r="I4" s="82"/>
-      <c r="J4" s="82"/>
-      <c r="K4" s="81"/>
-      <c r="L4" s="82"/>
-      <c r="M4" s="82"/>
-      <c r="N4" s="81"/>
-      <c r="O4" s="82"/>
-      <c r="P4" s="82"/>
-      <c r="Q4" s="81"/>
-      <c r="R4" s="82"/>
-      <c r="S4" s="82"/>
-      <c r="T4" s="81"/>
-      <c r="U4" s="82"/>
-      <c r="V4" s="82"/>
-      <c r="W4" s="81"/>
-      <c r="X4" s="82"/>
-      <c r="Y4" s="82"/>
-      <c r="Z4" s="81"/>
-      <c r="AA4" s="82"/>
-      <c r="AB4" s="82"/>
-      <c r="AC4" s="81"/>
-      <c r="AD4" s="82"/>
-      <c r="AE4" s="82"/>
-      <c r="AF4" s="81"/>
-      <c r="AG4" s="82"/>
-      <c r="AH4" s="82"/>
-      <c r="AI4" s="81"/>
-      <c r="AJ4" s="82"/>
-      <c r="AK4" s="82"/>
-      <c r="AL4" s="81"/>
-      <c r="AM4" s="82"/>
-      <c r="AN4" s="82"/>
-      <c r="AO4" s="81"/>
-      <c r="AP4" s="82"/>
-      <c r="AQ4" s="82"/>
-      <c r="AR4" s="81"/>
-      <c r="AS4" s="82"/>
-      <c r="AT4" s="82"/>
-      <c r="AU4" s="81"/>
-      <c r="AV4" s="82"/>
-      <c r="AW4" s="82"/>
-      <c r="AX4" s="81"/>
-      <c r="AY4" s="82"/>
-      <c r="AZ4" s="82"/>
-      <c r="BA4" s="81"/>
-      <c r="BB4" s="82"/>
-      <c r="BC4" s="82"/>
-      <c r="BD4" s="81"/>
-      <c r="BE4" s="82"/>
-      <c r="BF4" s="82"/>
-      <c r="BG4" s="81"/>
-      <c r="BH4" s="82"/>
-      <c r="BI4" s="82"/>
-      <c r="BJ4" s="81"/>
-      <c r="BK4" s="82"/>
-      <c r="BL4" s="82"/>
+      <c r="H4" s="101"/>
+      <c r="I4" s="102"/>
+      <c r="J4" s="102"/>
+      <c r="K4" s="101"/>
+      <c r="L4" s="102"/>
+      <c r="M4" s="102"/>
+      <c r="N4" s="101"/>
+      <c r="O4" s="102"/>
+      <c r="P4" s="102"/>
+      <c r="Q4" s="101"/>
+      <c r="R4" s="102"/>
+      <c r="S4" s="102"/>
+      <c r="T4" s="101"/>
+      <c r="U4" s="102"/>
+      <c r="V4" s="102"/>
+      <c r="W4" s="101"/>
+      <c r="X4" s="102"/>
+      <c r="Y4" s="102"/>
+      <c r="Z4" s="101"/>
+      <c r="AA4" s="102"/>
+      <c r="AB4" s="102"/>
+      <c r="AC4" s="101"/>
+      <c r="AD4" s="102"/>
+      <c r="AE4" s="102"/>
+      <c r="AF4" s="101"/>
+      <c r="AG4" s="102"/>
+      <c r="AH4" s="102"/>
+      <c r="AI4" s="101"/>
+      <c r="AJ4" s="102"/>
+      <c r="AK4" s="102"/>
+      <c r="AL4" s="101"/>
+      <c r="AM4" s="102"/>
+      <c r="AN4" s="102"/>
+      <c r="AO4" s="101"/>
+      <c r="AP4" s="102"/>
+      <c r="AQ4" s="102"/>
+      <c r="AR4" s="101"/>
+      <c r="AS4" s="102"/>
+      <c r="AT4" s="102"/>
+      <c r="AU4" s="101"/>
+      <c r="AV4" s="102"/>
+      <c r="AW4" s="102"/>
+      <c r="AX4" s="101"/>
+      <c r="AY4" s="102"/>
+      <c r="AZ4" s="102"/>
+      <c r="BA4" s="101"/>
+      <c r="BB4" s="102"/>
+      <c r="BC4" s="102"/>
+      <c r="BD4" s="101"/>
+      <c r="BE4" s="102"/>
+      <c r="BF4" s="102"/>
+      <c r="BG4" s="101"/>
+      <c r="BH4" s="102"/>
+      <c r="BI4" s="102"/>
+      <c r="BJ4" s="101"/>
+      <c r="BK4" s="102"/>
+      <c r="BL4" s="102"/>
       <c r="BM4" s="5"/>
       <c r="BN4" s="5"/>
       <c r="BO4" s="5"/>
@@ -1457,76 +1460,76 @@
       <c r="DP4" s="5"/>
     </row>
     <row r="5" spans="2:120" ht="42" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B5" s="103" t="s">
+      <c r="B5" s="96" t="s">
         <v>86</v>
       </c>
       <c r="C5" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="D5" s="85">
+      <c r="D5" s="103">
         <f>DATE(2025,8,16)</f>
         <v>45885</v>
       </c>
-      <c r="E5" s="82"/>
-      <c r="F5" s="86"/>
-      <c r="G5" s="87"/>
-      <c r="H5" s="81"/>
-      <c r="I5" s="82"/>
-      <c r="J5" s="82"/>
-      <c r="K5" s="81"/>
-      <c r="L5" s="82"/>
-      <c r="M5" s="82"/>
-      <c r="N5" s="81"/>
-      <c r="O5" s="82"/>
-      <c r="P5" s="82"/>
-      <c r="Q5" s="81"/>
-      <c r="R5" s="82"/>
-      <c r="S5" s="82"/>
-      <c r="T5" s="81"/>
-      <c r="U5" s="82"/>
-      <c r="V5" s="82"/>
-      <c r="W5" s="81"/>
-      <c r="X5" s="82"/>
-      <c r="Y5" s="82"/>
-      <c r="Z5" s="81"/>
-      <c r="AA5" s="82"/>
-      <c r="AB5" s="82"/>
-      <c r="AC5" s="81"/>
-      <c r="AD5" s="82"/>
-      <c r="AE5" s="82"/>
-      <c r="AF5" s="81"/>
-      <c r="AG5" s="82"/>
-      <c r="AH5" s="82"/>
-      <c r="AI5" s="81"/>
-      <c r="AJ5" s="82"/>
-      <c r="AK5" s="82"/>
-      <c r="AL5" s="81"/>
-      <c r="AM5" s="82"/>
-      <c r="AN5" s="82"/>
-      <c r="AO5" s="81"/>
-      <c r="AP5" s="82"/>
-      <c r="AQ5" s="82"/>
-      <c r="AR5" s="81"/>
-      <c r="AS5" s="82"/>
-      <c r="AT5" s="82"/>
-      <c r="AU5" s="81"/>
-      <c r="AV5" s="82"/>
-      <c r="AW5" s="82"/>
-      <c r="AX5" s="81"/>
-      <c r="AY5" s="82"/>
-      <c r="AZ5" s="82"/>
-      <c r="BA5" s="81"/>
-      <c r="BB5" s="82"/>
-      <c r="BC5" s="82"/>
-      <c r="BD5" s="81"/>
-      <c r="BE5" s="82"/>
-      <c r="BF5" s="82"/>
-      <c r="BG5" s="81"/>
-      <c r="BH5" s="82"/>
-      <c r="BI5" s="82"/>
-      <c r="BJ5" s="81"/>
-      <c r="BK5" s="82"/>
-      <c r="BL5" s="82"/>
+      <c r="E5" s="102"/>
+      <c r="F5" s="104"/>
+      <c r="G5" s="105"/>
+      <c r="H5" s="101"/>
+      <c r="I5" s="102"/>
+      <c r="J5" s="102"/>
+      <c r="K5" s="101"/>
+      <c r="L5" s="102"/>
+      <c r="M5" s="102"/>
+      <c r="N5" s="101"/>
+      <c r="O5" s="102"/>
+      <c r="P5" s="102"/>
+      <c r="Q5" s="101"/>
+      <c r="R5" s="102"/>
+      <c r="S5" s="102"/>
+      <c r="T5" s="101"/>
+      <c r="U5" s="102"/>
+      <c r="V5" s="102"/>
+      <c r="W5" s="101"/>
+      <c r="X5" s="102"/>
+      <c r="Y5" s="102"/>
+      <c r="Z5" s="101"/>
+      <c r="AA5" s="102"/>
+      <c r="AB5" s="102"/>
+      <c r="AC5" s="101"/>
+      <c r="AD5" s="102"/>
+      <c r="AE5" s="102"/>
+      <c r="AF5" s="101"/>
+      <c r="AG5" s="102"/>
+      <c r="AH5" s="102"/>
+      <c r="AI5" s="101"/>
+      <c r="AJ5" s="102"/>
+      <c r="AK5" s="102"/>
+      <c r="AL5" s="101"/>
+      <c r="AM5" s="102"/>
+      <c r="AN5" s="102"/>
+      <c r="AO5" s="101"/>
+      <c r="AP5" s="102"/>
+      <c r="AQ5" s="102"/>
+      <c r="AR5" s="101"/>
+      <c r="AS5" s="102"/>
+      <c r="AT5" s="102"/>
+      <c r="AU5" s="101"/>
+      <c r="AV5" s="102"/>
+      <c r="AW5" s="102"/>
+      <c r="AX5" s="101"/>
+      <c r="AY5" s="102"/>
+      <c r="AZ5" s="102"/>
+      <c r="BA5" s="101"/>
+      <c r="BB5" s="102"/>
+      <c r="BC5" s="102"/>
+      <c r="BD5" s="101"/>
+      <c r="BE5" s="102"/>
+      <c r="BF5" s="102"/>
+      <c r="BG5" s="101"/>
+      <c r="BH5" s="102"/>
+      <c r="BI5" s="102"/>
+      <c r="BJ5" s="101"/>
+      <c r="BK5" s="102"/>
+      <c r="BL5" s="102"/>
       <c r="BM5" s="5"/>
       <c r="BN5" s="5"/>
       <c r="BO5" s="5"/>
@@ -1592,82 +1595,82 @@
       </c>
       <c r="E6" s="5"/>
       <c r="F6" s="5"/>
-      <c r="G6" s="83" t="s">
+      <c r="G6" s="106" t="s">
         <v>3</v>
       </c>
-      <c r="H6" s="84"/>
-      <c r="I6" s="84"/>
-      <c r="J6" s="84"/>
-      <c r="K6" s="84"/>
-      <c r="L6" s="84"/>
-      <c r="M6" s="84"/>
-      <c r="N6" s="83" t="s">
+      <c r="H6" s="107"/>
+      <c r="I6" s="107"/>
+      <c r="J6" s="107"/>
+      <c r="K6" s="107"/>
+      <c r="L6" s="107"/>
+      <c r="M6" s="107"/>
+      <c r="N6" s="106" t="s">
         <v>4</v>
       </c>
-      <c r="O6" s="84"/>
-      <c r="P6" s="84"/>
-      <c r="Q6" s="84"/>
-      <c r="R6" s="84"/>
-      <c r="S6" s="84"/>
-      <c r="T6" s="84"/>
-      <c r="U6" s="83" t="s">
+      <c r="O6" s="107"/>
+      <c r="P6" s="107"/>
+      <c r="Q6" s="107"/>
+      <c r="R6" s="107"/>
+      <c r="S6" s="107"/>
+      <c r="T6" s="107"/>
+      <c r="U6" s="106" t="s">
         <v>5</v>
       </c>
-      <c r="V6" s="84"/>
-      <c r="W6" s="84"/>
-      <c r="X6" s="84"/>
-      <c r="Y6" s="84"/>
-      <c r="Z6" s="84"/>
-      <c r="AA6" s="84"/>
-      <c r="AB6" s="83" t="s">
+      <c r="V6" s="107"/>
+      <c r="W6" s="107"/>
+      <c r="X6" s="107"/>
+      <c r="Y6" s="107"/>
+      <c r="Z6" s="107"/>
+      <c r="AA6" s="107"/>
+      <c r="AB6" s="106" t="s">
         <v>6</v>
       </c>
-      <c r="AC6" s="84"/>
-      <c r="AD6" s="84"/>
-      <c r="AE6" s="84"/>
-      <c r="AF6" s="84"/>
-      <c r="AG6" s="84"/>
-      <c r="AH6" s="84"/>
-      <c r="AI6" s="83" t="s">
+      <c r="AC6" s="107"/>
+      <c r="AD6" s="107"/>
+      <c r="AE6" s="107"/>
+      <c r="AF6" s="107"/>
+      <c r="AG6" s="107"/>
+      <c r="AH6" s="107"/>
+      <c r="AI6" s="106" t="s">
         <v>5</v>
       </c>
-      <c r="AJ6" s="84"/>
-      <c r="AK6" s="84"/>
-      <c r="AL6" s="84"/>
-      <c r="AM6" s="84"/>
-      <c r="AN6" s="84"/>
-      <c r="AO6" s="84"/>
-      <c r="AP6" s="83" t="s">
+      <c r="AJ6" s="107"/>
+      <c r="AK6" s="107"/>
+      <c r="AL6" s="107"/>
+      <c r="AM6" s="107"/>
+      <c r="AN6" s="107"/>
+      <c r="AO6" s="107"/>
+      <c r="AP6" s="106" t="s">
         <v>7</v>
       </c>
-      <c r="AQ6" s="84"/>
-      <c r="AR6" s="84"/>
-      <c r="AS6" s="84"/>
-      <c r="AT6" s="84"/>
-      <c r="AU6" s="84"/>
-      <c r="AV6" s="84"/>
-      <c r="AW6" s="83" t="s">
+      <c r="AQ6" s="107"/>
+      <c r="AR6" s="107"/>
+      <c r="AS6" s="107"/>
+      <c r="AT6" s="107"/>
+      <c r="AU6" s="107"/>
+      <c r="AV6" s="107"/>
+      <c r="AW6" s="106" t="s">
         <v>8</v>
       </c>
-      <c r="AX6" s="84"/>
-      <c r="AY6" s="84"/>
-      <c r="AZ6" s="84"/>
-      <c r="BA6" s="84"/>
-      <c r="BB6" s="84"/>
-      <c r="BC6" s="84"/>
-      <c r="BD6" s="83" t="s">
+      <c r="AX6" s="107"/>
+      <c r="AY6" s="107"/>
+      <c r="AZ6" s="107"/>
+      <c r="BA6" s="107"/>
+      <c r="BB6" s="107"/>
+      <c r="BC6" s="107"/>
+      <c r="BD6" s="106" t="s">
         <v>9</v>
       </c>
-      <c r="BE6" s="84"/>
-      <c r="BF6" s="84"/>
-      <c r="BG6" s="84"/>
-      <c r="BH6" s="84"/>
-      <c r="BI6" s="84"/>
-      <c r="BJ6" s="84"/>
-      <c r="BK6" s="83" t="s">
+      <c r="BE6" s="107"/>
+      <c r="BF6" s="107"/>
+      <c r="BG6" s="107"/>
+      <c r="BH6" s="107"/>
+      <c r="BI6" s="107"/>
+      <c r="BJ6" s="107"/>
+      <c r="BK6" s="106" t="s">
         <v>10</v>
       </c>
-      <c r="BL6" s="84"/>
+      <c r="BL6" s="107"/>
       <c r="BM6" s="11"/>
       <c r="BN6" s="11"/>
       <c r="BO6" s="11"/>
@@ -1730,7 +1733,7 @@
     <row r="7" spans="2:120" ht="14.4" x14ac:dyDescent="0.3">
       <c r="B7" s="12"/>
       <c r="C7" s="12"/>
-      <c r="D7" s="102" t="s">
+      <c r="D7" s="95" t="s">
         <v>85</v>
       </c>
       <c r="E7" s="12"/>
@@ -2420,7 +2423,7 @@
         <v>22</v>
       </c>
       <c r="C9" s="19"/>
-      <c r="D9" s="101" t="s">
+      <c r="D9" s="94" t="s">
         <v>83</v>
       </c>
       <c r="E9" s="20">
@@ -2772,7 +2775,7 @@
       <c r="C14" s="39" t="s">
         <v>31</v>
       </c>
-      <c r="D14" s="90" t="s">
+      <c r="D14" s="83" t="s">
         <v>74</v>
       </c>
       <c r="E14" s="40"/>
@@ -3007,7 +3010,7 @@
       <c r="BJ16" s="27"/>
     </row>
     <row r="17" spans="2:82" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="B17" s="92" t="s">
+      <c r="B17" s="85" t="s">
         <v>75</v>
       </c>
       <c r="C17" s="29" t="s">
@@ -3095,7 +3098,7 @@
       <c r="K18" s="27"/>
       <c r="N18" s="27"/>
       <c r="P18" s="27"/>
-      <c r="Q18" s="88"/>
+      <c r="Q18" s="81"/>
       <c r="R18" s="27"/>
       <c r="S18" s="31"/>
       <c r="T18" s="31"/>
@@ -3143,7 +3146,7 @@
       <c r="BJ18" s="27"/>
     </row>
     <row r="19" spans="2:82" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="B19" s="92" t="s">
+      <c r="B19" s="85" t="s">
         <v>76</v>
       </c>
       <c r="C19" s="29" t="s">
@@ -3232,8 +3235,8 @@
       <c r="P20" s="27"/>
       <c r="Q20" s="27"/>
       <c r="R20" s="27"/>
-      <c r="S20" s="89"/>
-      <c r="T20" s="89"/>
+      <c r="S20" s="82"/>
+      <c r="T20" s="82"/>
       <c r="V20" s="31"/>
       <c r="W20" s="31"/>
       <c r="X20" s="31"/>
@@ -3306,8 +3309,8 @@
       <c r="X21" s="31"/>
       <c r="Y21" s="31"/>
       <c r="Z21" s="31"/>
-      <c r="AA21" s="91"/>
-      <c r="AB21" s="89"/>
+      <c r="AA21" s="84"/>
+      <c r="AB21" s="82"/>
       <c r="AC21" s="32"/>
       <c r="AD21" s="32"/>
       <c r="AE21" s="32"/>
@@ -3376,11 +3379,11 @@
       <c r="X22" s="27"/>
       <c r="Y22" s="27"/>
       <c r="Z22" s="27"/>
-      <c r="AA22" s="89"/>
+      <c r="AA22" s="82"/>
       <c r="AC22" s="32"/>
-      <c r="AD22" s="91"/>
-      <c r="AE22" s="91"/>
-      <c r="AF22" s="91"/>
+      <c r="AD22" s="84"/>
+      <c r="AE22" s="84"/>
+      <c r="AF22" s="84"/>
       <c r="AG22" s="32"/>
       <c r="AH22" s="32"/>
       <c r="AI22" s="32"/>
@@ -3485,7 +3488,7 @@
       <c r="C24" s="44" t="s">
         <v>26</v>
       </c>
-      <c r="D24" s="97" t="s">
+      <c r="D24" s="90" t="s">
         <v>74</v>
       </c>
       <c r="E24" s="45"/>
@@ -3622,7 +3625,7 @@
       <c r="B26" s="46" t="s">
         <v>44</v>
       </c>
-      <c r="C26" s="94" t="s">
+      <c r="C26" s="87" t="s">
         <v>28</v>
       </c>
       <c r="D26" s="29">
@@ -3693,7 +3696,7 @@
       <c r="B27" s="46" t="s">
         <v>45</v>
       </c>
-      <c r="C27" s="94" t="s">
+      <c r="C27" s="87" t="s">
         <v>28</v>
       </c>
       <c r="D27" s="29">
@@ -3738,9 +3741,9 @@
       <c r="AM27" s="32"/>
       <c r="AN27" s="32"/>
       <c r="AO27" s="32"/>
-      <c r="AR27" s="89"/>
-      <c r="AS27" s="89"/>
-      <c r="AT27" s="89"/>
+      <c r="AR27" s="82"/>
+      <c r="AS27" s="82"/>
+      <c r="AT27" s="82"/>
       <c r="AU27" s="31"/>
       <c r="AV27" s="31"/>
       <c r="AW27" s="31"/>
@@ -3808,11 +3811,11 @@
       <c r="AN28" s="32"/>
       <c r="AO28" s="32"/>
       <c r="AR28" s="32"/>
-      <c r="AS28" s="89"/>
-      <c r="AT28" s="89"/>
-      <c r="AU28" s="89"/>
-      <c r="AV28" s="89"/>
-      <c r="AW28" s="89"/>
+      <c r="AS28" s="82"/>
+      <c r="AT28" s="82"/>
+      <c r="AU28" s="82"/>
+      <c r="AV28" s="82"/>
+      <c r="AW28" s="82"/>
       <c r="AX28" s="31"/>
       <c r="AY28" s="31"/>
       <c r="AZ28" s="31"/>
@@ -3879,11 +3882,11 @@
       <c r="AR29" s="32"/>
       <c r="AS29" s="32"/>
       <c r="AT29" s="32"/>
-      <c r="AU29" s="89"/>
-      <c r="AV29" s="89"/>
-      <c r="AY29" s="89"/>
-      <c r="AZ29" s="89"/>
-      <c r="BA29" s="89"/>
+      <c r="AU29" s="82"/>
+      <c r="AV29" s="82"/>
+      <c r="AY29" s="82"/>
+      <c r="AZ29" s="82"/>
+      <c r="BA29" s="82"/>
       <c r="BB29" s="31"/>
       <c r="BC29" s="31"/>
       <c r="BD29" s="31"/>
@@ -3948,14 +3951,14 @@
       <c r="AT30" s="32"/>
       <c r="AU30" s="32"/>
       <c r="AV30" s="32"/>
-      <c r="AW30" s="89"/>
-      <c r="AX30" s="89"/>
-      <c r="AY30" s="89"/>
-      <c r="AZ30" s="89"/>
-      <c r="BA30" s="89"/>
-      <c r="BB30" s="89"/>
-      <c r="BC30" s="89"/>
-      <c r="BD30" s="89"/>
+      <c r="AW30" s="82"/>
+      <c r="AX30" s="82"/>
+      <c r="AY30" s="82"/>
+      <c r="AZ30" s="82"/>
+      <c r="BA30" s="82"/>
+      <c r="BB30" s="82"/>
+      <c r="BC30" s="82"/>
+      <c r="BD30" s="82"/>
       <c r="BE30" s="31"/>
       <c r="BF30" s="31"/>
       <c r="BH30" s="27"/>
@@ -3966,7 +3969,7 @@
       <c r="B31" s="46" t="s">
         <v>77</v>
       </c>
-      <c r="C31" s="94" t="s">
+      <c r="C31" s="87" t="s">
         <v>28</v>
       </c>
       <c r="D31" s="29">
@@ -4018,21 +4021,21 @@
       <c r="AV31" s="32"/>
       <c r="AW31" s="32"/>
       <c r="AX31" s="32"/>
-      <c r="AY31" s="89"/>
-      <c r="AZ31" s="89"/>
-      <c r="BA31" s="89"/>
-      <c r="BB31" s="89"/>
-      <c r="BC31" s="89"/>
-      <c r="BD31" s="89"/>
-      <c r="BE31" s="89"/>
-      <c r="BF31" s="89"/>
+      <c r="AY31" s="82"/>
+      <c r="AZ31" s="82"/>
+      <c r="BA31" s="82"/>
+      <c r="BB31" s="82"/>
+      <c r="BC31" s="82"/>
+      <c r="BD31" s="82"/>
+      <c r="BE31" s="82"/>
+      <c r="BF31" s="82"/>
       <c r="BG31" s="31"/>
       <c r="BH31" s="31"/>
       <c r="BI31" s="31"/>
       <c r="CD31" s="32"/>
     </row>
     <row r="32" spans="2:82" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="B32" s="93" t="s">
+      <c r="B32" s="86" t="s">
         <v>78</v>
       </c>
       <c r="C32" s="29" t="s">
@@ -4100,13 +4103,13 @@
       <c r="BG32" s="27"/>
       <c r="BH32" s="27"/>
       <c r="BI32" s="27"/>
-      <c r="BJ32" s="95"/>
-      <c r="BK32" s="95"/>
-      <c r="BL32" s="95"/>
-      <c r="BM32" s="95"/>
+      <c r="BJ32" s="88"/>
+      <c r="BK32" s="88"/>
+      <c r="BL32" s="88"/>
+      <c r="BM32" s="88"/>
     </row>
     <row r="33" spans="2:92" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="B33" s="93" t="s">
+      <c r="B33" s="86" t="s">
         <v>60</v>
       </c>
       <c r="C33" s="29" t="s">
@@ -4175,7 +4178,7 @@
       <c r="BH33" s="27"/>
       <c r="BI33" s="27"/>
       <c r="BJ33" s="27"/>
-      <c r="BN33" s="96"/>
+      <c r="BN33" s="89"/>
     </row>
     <row r="34" spans="2:92" ht="14.4" x14ac:dyDescent="0.3">
       <c r="B34" s="34" t="s">
@@ -4256,7 +4259,7 @@
       <c r="C35" s="50" t="s">
         <v>52</v>
       </c>
-      <c r="D35" s="99" t="s">
+      <c r="D35" s="92" t="s">
         <v>80</v>
       </c>
       <c r="E35" s="51"/>
@@ -4311,7 +4314,7 @@
       <c r="BB35" s="27"/>
       <c r="BC35" s="27"/>
       <c r="BJ35" s="27"/>
-      <c r="BQ35" s="89"/>
+      <c r="BQ35" s="82"/>
     </row>
     <row r="36" spans="2:92" ht="14.4" x14ac:dyDescent="0.3">
       <c r="B36" s="52" t="s">
@@ -4392,7 +4395,7 @@
         <v>54</v>
       </c>
       <c r="C37" s="29" t="s">
-        <v>52</v>
+        <v>87</v>
       </c>
       <c r="D37" s="29">
         <v>5</v>
@@ -4470,7 +4473,7 @@
         <v>55</v>
       </c>
       <c r="C38" s="29" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="D38" s="29">
         <v>2</v>
@@ -4685,7 +4688,7 @@
       <c r="CD40" s="55"/>
     </row>
     <row r="41" spans="2:92" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="B41" s="98" t="s">
+      <c r="B41" s="91" t="s">
         <v>79</v>
       </c>
       <c r="C41" s="29" t="s">
@@ -4999,7 +5002,7 @@
         <v>62</v>
       </c>
       <c r="C46" s="19"/>
-      <c r="D46" s="101" t="s">
+      <c r="D46" s="94" t="s">
         <v>84</v>
       </c>
       <c r="E46" s="57"/>
@@ -5020,7 +5023,7 @@
       <c r="B48" s="46" t="s">
         <v>44</v>
       </c>
-      <c r="C48" s="94" t="s">
+      <c r="C48" s="87" t="s">
         <v>65</v>
       </c>
       <c r="D48" s="29">
@@ -5110,7 +5113,7 @@
       <c r="B52" s="46" t="s">
         <v>69</v>
       </c>
-      <c r="C52" s="94" t="s">
+      <c r="C52" s="87" t="s">
         <v>28</v>
       </c>
       <c r="D52" s="29">
@@ -5127,7 +5130,7 @@
       <c r="B53" s="46" t="s">
         <v>70</v>
       </c>
-      <c r="C53" s="107" t="s">
+      <c r="C53" s="100" t="s">
         <v>28</v>
       </c>
       <c r="D53" s="29">
@@ -5156,20 +5159,20 @@
       <c r="CY54" s="55"/>
     </row>
     <row r="55" spans="2:120" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="B55" s="105" t="s">
+      <c r="B55" s="98" t="s">
         <v>72</v>
       </c>
       <c r="C55" s="65"/>
-      <c r="D55" s="100" t="s">
+      <c r="D55" s="93" t="s">
         <v>82</v>
       </c>
       <c r="E55" s="66"/>
     </row>
     <row r="56" spans="2:120" ht="29.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B56" s="104" t="s">
+      <c r="B56" s="97" t="s">
         <v>81</v>
       </c>
-      <c r="C56" s="106" t="s">
+      <c r="C56" s="99" t="s">
         <v>28</v>
       </c>
       <c r="D56" s="29">
@@ -5546,6 +5549,58 @@
     </row>
   </sheetData>
   <mergeCells count="68">
+    <mergeCell ref="AR5:AT5"/>
+    <mergeCell ref="AU5:AW5"/>
+    <mergeCell ref="W5:Y5"/>
+    <mergeCell ref="Z5:AB5"/>
+    <mergeCell ref="AC5:AE5"/>
+    <mergeCell ref="AF5:AH5"/>
+    <mergeCell ref="AI5:AK5"/>
+    <mergeCell ref="AL5:AN5"/>
+    <mergeCell ref="AO5:AQ5"/>
+    <mergeCell ref="BD6:BJ6"/>
+    <mergeCell ref="BK6:BL6"/>
+    <mergeCell ref="G6:M6"/>
+    <mergeCell ref="N6:T6"/>
+    <mergeCell ref="U6:AA6"/>
+    <mergeCell ref="AB6:AH6"/>
+    <mergeCell ref="AI6:AO6"/>
+    <mergeCell ref="AP6:AV6"/>
+    <mergeCell ref="AW6:BC6"/>
+    <mergeCell ref="AX3:AZ3"/>
+    <mergeCell ref="BA3:BC3"/>
+    <mergeCell ref="BD3:BF3"/>
+    <mergeCell ref="BG3:BI3"/>
+    <mergeCell ref="BJ3:BL3"/>
+    <mergeCell ref="AR3:AT3"/>
+    <mergeCell ref="AU3:AW3"/>
+    <mergeCell ref="H3:J3"/>
+    <mergeCell ref="K3:M3"/>
+    <mergeCell ref="N3:P3"/>
+    <mergeCell ref="Q3:S3"/>
+    <mergeCell ref="T3:V3"/>
+    <mergeCell ref="W3:Y3"/>
+    <mergeCell ref="Z3:AB3"/>
+    <mergeCell ref="AC3:AE3"/>
+    <mergeCell ref="AF3:AH3"/>
+    <mergeCell ref="AI3:AK3"/>
+    <mergeCell ref="AL3:AN3"/>
+    <mergeCell ref="AO3:AQ3"/>
+    <mergeCell ref="AC4:AE4"/>
+    <mergeCell ref="AF4:AH4"/>
+    <mergeCell ref="AI4:AK4"/>
+    <mergeCell ref="AL4:AN4"/>
+    <mergeCell ref="AO4:AQ4"/>
+    <mergeCell ref="H4:J4"/>
+    <mergeCell ref="K4:M4"/>
+    <mergeCell ref="N4:P4"/>
+    <mergeCell ref="Q4:S4"/>
+    <mergeCell ref="T4:V4"/>
+    <mergeCell ref="D5:E5"/>
+    <mergeCell ref="F5:G5"/>
+    <mergeCell ref="H5:J5"/>
+    <mergeCell ref="K5:M5"/>
+    <mergeCell ref="N5:P5"/>
     <mergeCell ref="BJ4:BL4"/>
     <mergeCell ref="AX5:AZ5"/>
     <mergeCell ref="BA5:BC5"/>
@@ -5562,58 +5617,6 @@
     <mergeCell ref="AU4:AW4"/>
     <mergeCell ref="W4:Y4"/>
     <mergeCell ref="Z4:AB4"/>
-    <mergeCell ref="D5:E5"/>
-    <mergeCell ref="F5:G5"/>
-    <mergeCell ref="H5:J5"/>
-    <mergeCell ref="K5:M5"/>
-    <mergeCell ref="N5:P5"/>
-    <mergeCell ref="H4:J4"/>
-    <mergeCell ref="K4:M4"/>
-    <mergeCell ref="N4:P4"/>
-    <mergeCell ref="Q4:S4"/>
-    <mergeCell ref="T4:V4"/>
-    <mergeCell ref="AC4:AE4"/>
-    <mergeCell ref="AF4:AH4"/>
-    <mergeCell ref="AI4:AK4"/>
-    <mergeCell ref="AL4:AN4"/>
-    <mergeCell ref="AO4:AQ4"/>
-    <mergeCell ref="AR3:AT3"/>
-    <mergeCell ref="AU3:AW3"/>
-    <mergeCell ref="H3:J3"/>
-    <mergeCell ref="K3:M3"/>
-    <mergeCell ref="N3:P3"/>
-    <mergeCell ref="Q3:S3"/>
-    <mergeCell ref="T3:V3"/>
-    <mergeCell ref="W3:Y3"/>
-    <mergeCell ref="Z3:AB3"/>
-    <mergeCell ref="AC3:AE3"/>
-    <mergeCell ref="AF3:AH3"/>
-    <mergeCell ref="AI3:AK3"/>
-    <mergeCell ref="AL3:AN3"/>
-    <mergeCell ref="AO3:AQ3"/>
-    <mergeCell ref="AX3:AZ3"/>
-    <mergeCell ref="BA3:BC3"/>
-    <mergeCell ref="BD3:BF3"/>
-    <mergeCell ref="BG3:BI3"/>
-    <mergeCell ref="BJ3:BL3"/>
-    <mergeCell ref="BD6:BJ6"/>
-    <mergeCell ref="BK6:BL6"/>
-    <mergeCell ref="G6:M6"/>
-    <mergeCell ref="N6:T6"/>
-    <mergeCell ref="U6:AA6"/>
-    <mergeCell ref="AB6:AH6"/>
-    <mergeCell ref="AI6:AO6"/>
-    <mergeCell ref="AP6:AV6"/>
-    <mergeCell ref="AW6:BC6"/>
-    <mergeCell ref="AR5:AT5"/>
-    <mergeCell ref="AU5:AW5"/>
-    <mergeCell ref="W5:Y5"/>
-    <mergeCell ref="Z5:AB5"/>
-    <mergeCell ref="AC5:AE5"/>
-    <mergeCell ref="AF5:AH5"/>
-    <mergeCell ref="AI5:AK5"/>
-    <mergeCell ref="AL5:AN5"/>
-    <mergeCell ref="AO5:AQ5"/>
   </mergeCells>
   <conditionalFormatting sqref="B5">
     <cfRule type="notContainsBlanks" dxfId="0" priority="1">

</xml_diff>